<commit_message>
Fix Product 5.1 Home weekly summary
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R4c1d5f850a174465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R1fb0230e481f498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rc52a2baeea5d4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R0c4f8b8aa6254f0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R4d91a9a3bcaa4448"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rac0a549c39824c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R5fa30f20c12549ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R008d1ba3ae5b4ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R6b7a1941031a451f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rd15fcc6bef634966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R2724018acddd4291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R03d1195022ca452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R8f003d884a9c4ebd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R6e10d6a6f24748f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R1e9f62a14bd141c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rad9ea3b3d76c46a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rb9eca20c846b45d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R736859a653864a3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R08b317e8bf234b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Ra628d3a6868a48d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R8d26e7fb23de485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R115db8a476074979"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +67,27 @@
       <x:color rgb="FF5F6368"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF5F6368"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:color rgb="FF5F6368"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="40">
+  <x:fills count="51">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -265,6 +284,61 @@
         <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B8043"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F8F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FBFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F3F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8F9FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE8B2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFAF0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -273,7 +347,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="157">
+  <x:cellXfs count="179">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -681,6 +755,72 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -850,17 +990,17 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18" customHeight="1">
-      <x:c r="A1" s="134" t="str">
+      <x:c r="A1" s="157" t="str">
         <x:v>SIMS-Blog-Manager  Home</x:v>
       </x:c>
-      <x:c r="B1" s="134"/>
-      <x:c r="C1" s="134"/>
-      <x:c r="D1" s="134"/>
-      <x:c r="E1" s="134"/>
-      <x:c r="F1" s="134"/>
-      <x:c r="G1" s="134"/>
-      <x:c r="H1" s="135" t="str">
-        <x:v>v5.1.0</x:v>
+      <x:c r="B1" s="157"/>
+      <x:c r="C1" s="157"/>
+      <x:c r="D1" s="157"/>
+      <x:c r="E1" s="157"/>
+      <x:c r="F1" s="157"/>
+      <x:c r="G1" s="157"/>
+      <x:c r="H1" s="158" t="str">
+        <x:v>v5.1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -908,70 +1048,70 @@
       <x:c r="H4" s="36"/>
     </x:row>
     <x:row r="5" ht="18" customHeight="1">
-      <x:c r="A5" s="137" t="str">
+      <x:c r="A5" s="159" t="str">
         <x:v>記事ランクのまとめ</x:v>
       </x:c>
-      <x:c r="B5" s="137"/>
-      <x:c r="C5" s="137"/>
-      <x:c r="D5" s="137"/>
-      <x:c r="E5" s="137"/>
-      <x:c r="F5" s="137"/>
-      <x:c r="G5" s="137"/>
-      <x:c r="H5" s="137"/>
+      <x:c r="B5" s="159"/>
+      <x:c r="C5" s="159"/>
+      <x:c r="D5" s="159"/>
+      <x:c r="E5" s="159"/>
+      <x:c r="F5" s="159"/>
+      <x:c r="G5" s="159"/>
+      <x:c r="H5" s="159"/>
     </x:row>
     <x:row r="6" ht="18" customHeight="1">
-      <x:c r="A6" s="138" t="str">
+      <x:c r="A6" s="160" t="str">
         <x:v>🏆 エース</x:v>
       </x:c>
-      <x:c r="B6" s="138"/>
-      <x:c r="C6" s="138" t="str">
+      <x:c r="B6" s="160"/>
+      <x:c r="C6" s="160" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="D6" s="138"/>
-      <x:c r="E6" s="139" t="str">
+      <x:c r="D6" s="160"/>
+      <x:c r="E6" s="161" t="str">
         <x:v>🌱 育成</x:v>
       </x:c>
-      <x:c r="F6" s="139"/>
-      <x:c r="G6" s="139" t="str">
+      <x:c r="F6" s="161"/>
+      <x:c r="G6" s="161" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="H6" s="139"/>
+      <x:c r="H6" s="161"/>
     </x:row>
     <x:row r="7" ht="18" customHeight="1">
-      <x:c r="A7" s="138" t="str">
+      <x:c r="A7" s="160" t="str">
         <x:v>✅ 安定</x:v>
       </x:c>
-      <x:c r="B7" s="138"/>
-      <x:c r="C7" s="138" t="str">
+      <x:c r="B7" s="160"/>
+      <x:c r="C7" s="160" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="D7" s="138"/>
-      <x:c r="E7" s="139" t="str">
+      <x:c r="D7" s="160"/>
+      <x:c r="E7" s="161" t="str">
         <x:v>⚠️ 迷走</x:v>
       </x:c>
-      <x:c r="F7" s="139"/>
-      <x:c r="G7" s="139" t="str">
+      <x:c r="F7" s="161"/>
+      <x:c r="G7" s="161" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="H7" s="139"/>
+      <x:c r="H7" s="161"/>
     </x:row>
     <x:row r="8" ht="18" customHeight="1">
-      <x:c r="A8" s="138" t="str">
+      <x:c r="A8" s="160" t="str">
         <x:v>📈 成長</x:v>
       </x:c>
-      <x:c r="B8" s="138"/>
-      <x:c r="C8" s="138" t="str">
+      <x:c r="B8" s="160"/>
+      <x:c r="C8" s="160" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="D8" s="138"/>
-      <x:c r="E8" s="139" t="str">
+      <x:c r="D8" s="160"/>
+      <x:c r="E8" s="161" t="str">
         <x:v>❓ 未取得</x:v>
       </x:c>
-      <x:c r="F8" s="139"/>
-      <x:c r="G8" s="139" t="str">
+      <x:c r="F8" s="161"/>
+      <x:c r="G8" s="161" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="H8" s="139"/>
+      <x:c r="H8" s="161"/>
     </x:row>
     <x:row r="9" ht="18" customHeight="1">
       <x:c r="A9" s="116"/>
@@ -984,38 +1124,38 @@
       <x:c r="H9" s="115"/>
     </x:row>
     <x:row r="10" ht="18" customHeight="1">
-      <x:c r="A10" s="140" t="str">
+      <x:c r="A10" s="162" t="str">
         <x:v>今日のメッセージ</x:v>
       </x:c>
-      <x:c r="B10" s="140"/>
-      <x:c r="C10" s="140"/>
-      <x:c r="D10" s="140"/>
-      <x:c r="E10" s="140"/>
-      <x:c r="F10" s="140"/>
-      <x:c r="G10" s="140"/>
-      <x:c r="H10" s="140"/>
+      <x:c r="B10" s="162"/>
+      <x:c r="C10" s="162"/>
+      <x:c r="D10" s="162"/>
+      <x:c r="E10" s="162"/>
+      <x:c r="F10" s="162"/>
+      <x:c r="G10" s="162"/>
+      <x:c r="H10" s="162"/>
     </x:row>
     <x:row r="11" ht="18" customHeight="1">
-      <x:c r="A11" s="141" t="str">
+      <x:c r="A11" s="164" t="str">
         <x:v>記事の育ち方と改善状況に合わせて表示します。</x:v>
       </x:c>
-      <x:c r="B11" s="141"/>
-      <x:c r="C11" s="141"/>
-      <x:c r="D11" s="141"/>
-      <x:c r="E11" s="141"/>
-      <x:c r="F11" s="141"/>
-      <x:c r="G11" s="141"/>
-      <x:c r="H11" s="141"/>
+      <x:c r="B11" s="164"/>
+      <x:c r="C11" s="164"/>
+      <x:c r="D11" s="164"/>
+      <x:c r="E11" s="164"/>
+      <x:c r="F11" s="164"/>
+      <x:c r="G11" s="164"/>
+      <x:c r="H11" s="164"/>
     </x:row>
     <x:row r="12" ht="18" customHeight="1">
-      <x:c r="A12" s="141"/>
-      <x:c r="B12" s="141"/>
-      <x:c r="C12" s="141"/>
-      <x:c r="D12" s="141"/>
-      <x:c r="E12" s="141"/>
-      <x:c r="F12" s="141"/>
-      <x:c r="G12" s="141"/>
-      <x:c r="H12" s="141"/>
+      <x:c r="A12" s="164"/>
+      <x:c r="B12" s="164"/>
+      <x:c r="C12" s="164"/>
+      <x:c r="D12" s="164"/>
+      <x:c r="E12" s="164"/>
+      <x:c r="F12" s="164"/>
+      <x:c r="G12" s="164"/>
+      <x:c r="H12" s="164"/>
     </x:row>
     <x:row r="13" ht="18" customHeight="1">
       <x:c r="A13" s="96"/>
@@ -1028,117 +1168,115 @@
       <x:c r="H13" s="96"/>
     </x:row>
     <x:row r="14" ht="18" customHeight="1">
-      <x:c r="A14" s="144" t="str">
+      <x:c r="A14" s="165" t="str">
         <x:v>改善状況</x:v>
       </x:c>
-      <x:c r="B14" s="144"/>
-      <x:c r="C14" s="144"/>
-      <x:c r="D14" s="144"/>
-      <x:c r="E14" s="137" t="str">
+      <x:c r="B14" s="165"/>
+      <x:c r="C14" s="165"/>
+      <x:c r="D14" s="165"/>
+      <x:c r="E14" s="159" t="str">
         <x:v>今週の取り組み</x:v>
       </x:c>
-      <x:c r="F14" s="137"/>
-      <x:c r="G14" s="137"/>
-      <x:c r="H14" s="137"/>
+      <x:c r="F14" s="159"/>
+      <x:c r="G14" s="159"/>
+      <x:c r="H14" s="159"/>
     </x:row>
     <x:row r="15" ht="18" customHeight="1">
       <x:c r="A15" s="145" t="str">
         <x:v>今日の改善</x:v>
       </x:c>
       <x:c r="B15" s="145"/>
-      <x:c r="C15" s="150" t="str">
+      <x:c r="C15" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="D15" s="150"/>
+      <x:c r="D15" s="166"/>
       <x:c r="E15" s="145" t="str">
         <x:v>今週改善した記事</x:v>
       </x:c>
       <x:c r="F15" s="145"/>
-      <x:c r="G15" s="150" t="str">
+      <x:c r="G15" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="H15" s="150"/>
+      <x:c r="H15" s="166"/>
     </x:row>
     <x:row r="16" ht="18" customHeight="1">
       <x:c r="A16" s="145" t="str">
         <x:v>改善中</x:v>
       </x:c>
       <x:c r="B16" s="145"/>
-      <x:c r="C16" s="150" t="str">
+      <x:c r="C16" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="D16" s="150"/>
+      <x:c r="D16" s="166"/>
       <x:c r="E16" s="145" t="str">
         <x:v>改善推移確認中</x:v>
       </x:c>
       <x:c r="F16" s="145"/>
-      <x:c r="G16" s="150" t="str">
+      <x:c r="G16" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="H16" s="150"/>
+      <x:c r="H16" s="166"/>
     </x:row>
     <x:row r="17" ht="18" customHeight="1">
       <x:c r="A17" s="145" t="str">
         <x:v>改善推移確認中</x:v>
       </x:c>
       <x:c r="B17" s="145"/>
-      <x:c r="C17" s="150" t="str">
+      <x:c r="C17" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="D17" s="150"/>
+      <x:c r="D17" s="166"/>
       <x:c r="E17" s="145" t="str">
         <x:v>改善確認完了</x:v>
       </x:c>
       <x:c r="F17" s="145"/>
-      <x:c r="G17" s="150" t="str">
+      <x:c r="G17" s="166" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="H17" s="150"/>
+      <x:c r="H17" s="166"/>
     </x:row>
     <x:row r="18" ht="18" customHeight="1">
       <x:c r="A18" s="148" t="str">
         <x:v>未取得記事</x:v>
       </x:c>
       <x:c r="B18" s="148"/>
-      <x:c r="C18" s="112" t="str">
+      <x:c r="C18" s="167" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="D18" s="112"/>
+      <x:c r="D18" s="167"/>
       <x:c r="E18" s="149" t="str">
         <x:v>改善候補</x:v>
       </x:c>
       <x:c r="F18" s="149"/>
-      <x:c r="G18" s="112" t="str">
+      <x:c r="G18" s="167" t="str">
         <x:v>0件</x:v>
       </x:c>
-      <x:c r="H18" s="112"/>
+      <x:c r="H18" s="167"/>
     </x:row>
     <x:row r="19" ht="18" customHeight="1">
-      <x:c r="A19" s="36"/>
-      <x:c r="B19" s="36"/>
-      <x:c r="C19" s="36"/>
-      <x:c r="D19" s="36"/>
-      <x:c r="E19" s="36"/>
-      <x:c r="F19" s="36"/>
-      <x:c r="G19" s="36"/>
-      <x:c r="H19" s="36"/>
+      <x:c r="A19" s="170" t="str">
+        <x:v>※未取得記事：Search Consoleから一時的にデータを取得できなかった記事などです。記事が削除されたことを意味するものではありません。</x:v>
+      </x:c>
+      <x:c r="B19" s="170"/>
+      <x:c r="C19" s="170"/>
+      <x:c r="D19" s="170"/>
+      <x:c r="E19" s="170"/>
+      <x:c r="F19" s="170"/>
+      <x:c r="G19" s="170"/>
+      <x:c r="H19" s="170"/>
     </x:row>
     <x:row r="20" ht="18" customHeight="1">
-      <x:c r="A20" s="151" t="str">
-        <x:v>今週のアドバイス</x:v>
-      </x:c>
-      <x:c r="B20" s="151"/>
-      <x:c r="C20" s="151"/>
-      <x:c r="D20" s="151"/>
-      <x:c r="E20" s="151"/>
-      <x:c r="F20" s="151"/>
-      <x:c r="G20" s="151"/>
-      <x:c r="H20" s="151"/>
+      <x:c r="A20" s="170"/>
+      <x:c r="B20" s="170"/>
+      <x:c r="C20" s="170"/>
+      <x:c r="D20" s="170"/>
+      <x:c r="E20" s="170"/>
+      <x:c r="F20" s="170"/>
+      <x:c r="G20" s="170"/>
+      <x:c r="H20" s="170"/>
     </x:row>
     <x:row r="21" ht="18" customHeight="1">
-      <x:c r="A21" s="152" t="str">
-        <x:v>今週の取り組みに合わせて、次の作業を案内します。</x:v>
-      </x:c>
+      <x:c r="A21" s="152"/>
       <x:c r="B21" s="152"/>
       <x:c r="C21" s="152"/>
       <x:c r="D21" s="152"/>
@@ -1148,41 +1286,41 @@
       <x:c r="H21" s="152"/>
     </x:row>
     <x:row r="22" ht="18" customHeight="1">
-      <x:c r="A22" s="153"/>
-      <x:c r="B22" s="153"/>
-      <x:c r="C22" s="153"/>
-      <x:c r="D22" s="153"/>
-      <x:c r="E22" s="153"/>
-      <x:c r="F22" s="153"/>
-      <x:c r="G22" s="153"/>
-      <x:c r="H22" s="153"/>
+      <x:c r="A22" s="172" t="str">
+        <x:v>今週のアドバイス</x:v>
+      </x:c>
+      <x:c r="B22" s="172"/>
+      <x:c r="C22" s="172"/>
+      <x:c r="D22" s="172"/>
+      <x:c r="E22" s="172"/>
+      <x:c r="F22" s="172"/>
+      <x:c r="G22" s="172"/>
+      <x:c r="H22" s="172"/>
     </x:row>
     <x:row r="23" ht="18" customHeight="1">
-      <x:c r="A23" s="99" t="str">
-        <x:v>※未取得記事：Search Consoleから一時的にデータを取得できなかった記事などです。記事が削除されたことを意味するものではありません。</x:v>
-      </x:c>
-      <x:c r="B23" s="99"/>
-      <x:c r="C23" s="99"/>
-      <x:c r="D23" s="99"/>
-      <x:c r="E23" s="99"/>
-      <x:c r="F23" s="99"/>
-      <x:c r="G23" s="99"/>
-      <x:c r="H23" s="99"/>
+      <x:c r="A23" s="175" t="str">
+        <x:v>今週の取り組みに合わせて、次の作業を案内します。</x:v>
+      </x:c>
+      <x:c r="B23" s="175"/>
+      <x:c r="C23" s="175"/>
+      <x:c r="D23" s="175"/>
+      <x:c r="E23" s="175"/>
+      <x:c r="F23" s="175"/>
+      <x:c r="G23" s="175"/>
+      <x:c r="H23" s="175"/>
     </x:row>
     <x:row r="24" ht="18" customHeight="1">
-      <x:c r="A24" s="154"/>
-      <x:c r="B24" s="154"/>
-      <x:c r="C24" s="154"/>
-      <x:c r="D24" s="154"/>
-      <x:c r="E24" s="154"/>
-      <x:c r="F24" s="154"/>
-      <x:c r="G24" s="154"/>
-      <x:c r="H24" s="154"/>
+      <x:c r="A24" s="176"/>
+      <x:c r="B24" s="176"/>
+      <x:c r="C24" s="176"/>
+      <x:c r="D24" s="176"/>
+      <x:c r="E24" s="176"/>
+      <x:c r="F24" s="176"/>
+      <x:c r="G24" s="176"/>
+      <x:c r="H24" s="176"/>
     </x:row>
     <x:row r="25" ht="18" customHeight="1">
-      <x:c r="A25" s="36" t="str">
-        <x:v>処理状況</x:v>
-      </x:c>
+      <x:c r="A25" s="36"/>
       <x:c r="B25" s="36"/>
       <x:c r="C25" s="36"/>
       <x:c r="D25" s="36"/>
@@ -1192,52 +1330,54 @@
       <x:c r="H25" s="36"/>
     </x:row>
     <x:row r="26" ht="18" customHeight="1">
-      <x:c r="A26" s="156" t="str">
+      <x:c r="A26" s="177" t="str">
+        <x:v>処理状況</x:v>
+      </x:c>
+      <x:c r="B26" s="177"/>
+      <x:c r="C26" s="177"/>
+      <x:c r="D26" s="177"/>
+      <x:c r="E26" s="177"/>
+      <x:c r="F26" s="177"/>
+      <x:c r="G26" s="177"/>
+      <x:c r="H26" s="177"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="178" t="str">
         <x:v>処理名</x:v>
       </x:c>
-      <x:c r="B26" s="156"/>
-      <x:c r="C26" s="156"/>
-      <x:c r="D26" s="156"/>
-      <x:c r="E26" s="156"/>
-      <x:c r="F26" s="156"/>
-      <x:c r="G26" s="156"/>
-      <x:c r="H26" s="156"/>
-    </x:row>
-    <x:row r="27" ht="18" customHeight="1">
-      <x:c r="A27" s="155" t="str">
+      <x:c r="B27" s="178"/>
+      <x:c r="C27" s="178"/>
+      <x:c r="D27" s="178"/>
+      <x:c r="E27" s="178"/>
+      <x:c r="F27" s="178"/>
+      <x:c r="G27" s="178"/>
+      <x:c r="H27" s="178"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="178" t="str">
         <x:v>開始時刻</x:v>
       </x:c>
-      <x:c r="B27" s="155"/>
-      <x:c r="C27" s="155"/>
-      <x:c r="D27" s="155" t="str">
+      <x:c r="B28" s="178"/>
+      <x:c r="C28" s="178"/>
+      <x:c r="D28" s="178" t="str">
         <x:v>処理結果</x:v>
       </x:c>
-      <x:c r="E27" s="155"/>
-      <x:c r="F27" s="155"/>
-      <x:c r="G27" s="155"/>
-      <x:c r="H27" s="155"/>
-    </x:row>
-    <x:row r="28" ht="18" customHeight="1">
-      <x:c r="A28" s="155" t="str">
+      <x:c r="E28" s="178"/>
+      <x:c r="F28" s="178"/>
+      <x:c r="G28" s="178"/>
+      <x:c r="H28" s="178"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="178" t="str">
         <x:v>お願い</x:v>
       </x:c>
-      <x:c r="B28" s="155"/>
-      <x:c r="C28" s="155"/>
-      <x:c r="D28" s="155"/>
-      <x:c r="E28" s="155"/>
-      <x:c r="F28" s="155"/>
-      <x:c r="G28" s="155"/>
-      <x:c r="H28" s="155"/>
-    </x:row>
-    <x:row r="29" ht="18" customHeight="1">
-      <x:c r="A29" s="155"/>
-      <x:c r="B29" s="155"/>
-      <x:c r="C29" s="155"/>
-      <x:c r="D29" s="155"/>
-      <x:c r="E29" s="155"/>
-      <x:c r="F29" s="155"/>
-      <x:c r="G29" s="155"/>
-      <x:c r="H29" s="155"/>
+      <x:c r="B29" s="178"/>
+      <x:c r="C29" s="178"/>
+      <x:c r="D29" s="178"/>
+      <x:c r="E29" s="178"/>
+      <x:c r="F29" s="178"/>
+      <x:c r="G29" s="178"/>
+      <x:c r="H29" s="178"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="28"/>
@@ -1341,6 +1481,9 @@
     <x:mergeCell ref="B28:C28"/>
     <x:mergeCell ref="E28:H28"/>
     <x:mergeCell ref="B29:H29"/>
+    <x:mergeCell ref="A19:H20"/>
+    <x:mergeCell ref="A22:H22"/>
+    <x:mergeCell ref="A23:H24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10088,7 +10231,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.1.0</x:v>
+        <x:v>5.1.1</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Reorganize Product 5.1 menus
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R03d1195022ca452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R8f003d884a9c4ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R6e10d6a6f24748f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R1e9f62a14bd141c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rad9ea3b3d76c46a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rb9eca20c846b45d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R736859a653864a3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R08b317e8bf234b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Ra628d3a6868a48d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R8d26e7fb23de485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R115db8a476074979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R3a037188697d41b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf6d487fb42ba486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R4176a1fdfd6c487d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R723a258d676948e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R3a1808ca7870455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Ra5eee99431584f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R9ac22396beb746e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rb35fd6ce1c144837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R447d9f1ffdd1484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Ra646c61eceeb44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Raaf9a4fa11eb44ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="12">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +86,13 @@
       <x:color rgb="FF5F6368"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF5F6368"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="51">
+  <x:fills count="52">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -339,6 +344,11 @@
         <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -347,7 +357,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="179">
+  <x:cellXfs count="188">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -822,6 +832,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1000,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.1.1</x:v>
+        <x:v>v5.1.2</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -1254,26 +1291,26 @@
       <x:c r="H18" s="167"/>
     </x:row>
     <x:row r="19" ht="18" customHeight="1">
-      <x:c r="A19" s="170" t="str">
+      <x:c r="A19" s="187" t="str">
         <x:v>※未取得記事：Search Consoleから一時的にデータを取得できなかった記事などです。記事が削除されたことを意味するものではありません。</x:v>
       </x:c>
-      <x:c r="B19" s="170"/>
-      <x:c r="C19" s="170"/>
-      <x:c r="D19" s="170"/>
-      <x:c r="E19" s="170"/>
-      <x:c r="F19" s="170"/>
-      <x:c r="G19" s="170"/>
-      <x:c r="H19" s="170"/>
+      <x:c r="B19" s="187"/>
+      <x:c r="C19" s="187"/>
+      <x:c r="D19" s="187"/>
+      <x:c r="E19" s="187"/>
+      <x:c r="F19" s="187"/>
+      <x:c r="G19" s="187"/>
+      <x:c r="H19" s="187"/>
     </x:row>
     <x:row r="20" ht="18" customHeight="1">
-      <x:c r="A20" s="170"/>
-      <x:c r="B20" s="170"/>
-      <x:c r="C20" s="170"/>
-      <x:c r="D20" s="170"/>
-      <x:c r="E20" s="170"/>
-      <x:c r="F20" s="170"/>
-      <x:c r="G20" s="170"/>
-      <x:c r="H20" s="170"/>
+      <x:c r="A20" s="187"/>
+      <x:c r="B20" s="187"/>
+      <x:c r="C20" s="187"/>
+      <x:c r="D20" s="187"/>
+      <x:c r="E20" s="187"/>
+      <x:c r="F20" s="187"/>
+      <x:c r="G20" s="187"/>
+      <x:c r="H20" s="187"/>
     </x:row>
     <x:row r="21" ht="18" customHeight="1">
       <x:c r="A21" s="152"/>
@@ -10231,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.1.1</x:v>
+        <x:v>5.1.2</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Fix Product 5.1 menus and history styling
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.1-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R3a037188697d41b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf6d487fb42ba486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R4176a1fdfd6c487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R723a258d676948e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R3a1808ca7870455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Ra5eee99431584f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R9ac22396beb746e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rb35fd6ce1c144837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R447d9f1ffdd1484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Ra646c61eceeb44ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Raaf9a4fa11eb44ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Re7304e4b1eb54346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R1dbf4bdd6b5e4bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R0616dd57ab534f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Rc10d6c113b184ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R9a6ad3cecc094336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R9f424033efd74e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rc6c8c246fbd74b64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R465d41b0826349be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Raf10992930d048a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R516ad02f137e4cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rdd5b684bca0841c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.1.2</x:v>
+        <x:v>v5.1.3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10268,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.1.2</x:v>
+        <x:v>5.1.3</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>